<commit_message>
Roll MGX/New Space to Q2'26 fund reporting; close EsyaSoft/Mena Mobile/VTVT open items; fix cashflow sign bug, missing-vehicle dashboard gap, and tooltip CSS clipping
</commit_message>
<xml_diff>
--- a/data/outputs/Tracker_Extract_Reconciled.xlsx
+++ b/data/outputs/Tracker_Extract_Reconciled.xlsx
@@ -12954,28 +12954,28 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>28252147.046175</v>
+        <v>47540482</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>1</v>
+        <v>1.1394</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Monthly Tracker (Valuation team)</t>
+          <t>ECB euro reference rate (EUR/USD, 30 Jun 2026)</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -12985,7 +12985,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Q1'26  capital account statement</t>
+          <t>Q2'26 Limited Partner Statement (NewSpace Capital Fund S.C.S., for G42 Investments AI Holding Limited)</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -13309,11 +13309,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>644147257.37</v>
+        <v>948484252</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -13325,7 +13325,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -13340,7 +13340,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Q4'25  capital account statement</t>
+          <t>Q2'26 capital account statement</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -13380,11 +13380,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>741856786</v>
+        <v>1180373331</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -13396,7 +13396,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -13411,7 +13411,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Q4'25  capital account statement</t>
+          <t>Q2'26 capital account statement</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -13522,11 +13522,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2025-09-30</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>41594050</v>
+        <v>62794035</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -13538,7 +13538,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2025-09-30</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -13553,7 +13553,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>MANUALLY ADDED - see repo memory for details. Re-add after every apply-reconciliation re-run.</t>
+          <t>Q2'26 capital account statement</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">

</xml_diff>